<commit_message>
Optimize Termux wake return flow
</commit_message>
<xml_diff>
--- a/docs/project-management/lukua-launcher-AI项目管理模板.xlsx
+++ b/docs/project-management/lukua-launcher-AI项目管理模板.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="Rc19281e0b1c146af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总表" sheetId="2" r:id="R79f28a4c178243d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发版检查" sheetId="3" r:id="R7037ec9425034238"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兼容性测试" sheetId="4" r:id="Rd05448d4a9ce4e6e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI协作记录" sheetId="5" r:id="R05f6683c07384936"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R0a9eb14720df4291"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总表" sheetId="2" r:id="R9383fa6503694b40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发版检查" sheetId="3" r:id="R77492ed9b2304fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兼容性测试" sheetId="4" r:id="R76644b2741ec42f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI协作记录" sheetId="5" r:id="Rb28bc6f2f7e04746"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -369,7 +369,7 @@
         <x:color rgb="FF14532D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -380,7 +380,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -391,7 +391,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -402,7 +402,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -413,7 +413,7 @@
         <x:color rgb="FF14532D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -424,7 +424,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -435,7 +435,7 @@
         <x:color rgb="FF14532D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -446,7 +446,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -457,7 +457,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -468,7 +468,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -479,7 +479,7 @@
         <x:color rgb="FF14532D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -490,7 +490,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -501,7 +501,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -512,7 +512,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -523,7 +523,7 @@
         <x:color rgb="FF14532D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -534,7 +534,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -545,7 +545,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -556,7 +556,7 @@
         <x:color rgb="FF14532D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFD9F2E3"/>
         </x:patternFill>
       </x:fill>
@@ -567,7 +567,7 @@
         <x:color rgb="FF7F1D1D"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE2E1"/>
         </x:patternFill>
       </x:fill>
@@ -578,7 +578,7 @@
         <x:color rgb="FF854D0E"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF4CC"/>
         </x:patternFill>
       </x:fill>
@@ -1162,7 +1162,7 @@
       </x:c>
       <x:c r="E11" s="56" t="n">
         <x:f>COUNTA('版本总表'!A6:A200)</x:f>
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1216,7 +1216,7 @@
       </x:c>
       <x:c r="E15" s="56" t="n">
         <x:f>COUNTA('兼容性测试'!A6:A300)</x:f>
-        <x:v>2</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16"/>
@@ -1854,19 +1854,43 @@
         <x:v>可作为当前基线版继续开发</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="55" t="str"/>
-      <x:c r="B6" s="55" t="str"/>
-      <x:c r="C6" s="55" t="str"/>
-      <x:c r="D6" s="55" t="str"/>
-      <x:c r="E6" s="55" t="str"/>
-      <x:c r="F6" s="55" t="str"/>
-      <x:c r="G6" s="55" t="str"/>
-      <x:c r="H6" s="55" t="str"/>
-      <x:c r="I6" s="55" t="str"/>
-      <x:c r="J6" s="55" t="str"/>
-      <x:c r="K6" s="55" t="str"/>
-      <x:c r="L6" s="55" t="str"/>
+    <x:row r="6" ht="72" hidden="0" customHeight="1">
+      <x:c r="A6" s="55" t="str">
+        <x:v>v0.9.1-beta5</x:v>
+      </x:c>
+      <x:c r="B6" s="55" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="C6" s="55" t="str">
+        <x:v>v0.9.1-beta4</x:v>
+      </x:c>
+      <x:c r="D6" s="55" t="str">
+        <x:v>beta</x:v>
+      </x:c>
+      <x:c r="E6" s="55" t="str">
+        <x:v>优化 Termux 唤醒与首次跳转返回体验</x:v>
+      </x:c>
+      <x:c r="F6" s="55" t="str">
+        <x:v>回前台按条件自动唤醒 Termux；按钮和首次引导改用可解释的唤醒结果；权限和诊断说明更清楚。</x:v>
+      </x:c>
+      <x:c r="G6" s="55" t="str">
+        <x:v>修复冷却中仍显示已唤醒、首启引导重复弹出、Termux 后台已放行仍提醒的问题。</x:v>
+      </x:c>
+      <x:c r="H6" s="55" t="str">
+        <x:v>本环境无在线 adb 设备，未做真机安装和前后台手动验证；不同系统省电策略仍需复测。</x:v>
+      </x:c>
+      <x:c r="I6" s="55" t="str">
+        <x:v>构建通过</x:v>
+      </x:c>
+      <x:c r="J6" s="55" t="str">
+        <x:v>构建通过，真机待测</x:v>
+      </x:c>
+      <x:c r="K6" s="55" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L6" s="55" t="str">
+        <x:v>发布为 prerelease，建议真机确认后继续作为主线。</x:v>
+      </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="55" t="str"/>
@@ -5222,35 +5246,83 @@
         <x:v>模板文件可直接复制重建，不影响 APK</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="55" t="str"/>
-      <x:c r="B6" s="55" t="str"/>
-      <x:c r="C6" s="55" t="str"/>
-      <x:c r="D6" s="55" t="str"/>
-      <x:c r="E6" s="55" t="str"/>
-      <x:c r="F6" s="55" t="str"/>
-      <x:c r="G6" s="55" t="str"/>
-      <x:c r="H6" s="55" t="str"/>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="55" t="str"/>
-      <x:c r="B7" s="55" t="str"/>
-      <x:c r="C7" s="55" t="str"/>
-      <x:c r="D7" s="55" t="str"/>
-      <x:c r="E7" s="55" t="str"/>
-      <x:c r="F7" s="55" t="str"/>
-      <x:c r="G7" s="55" t="str"/>
-      <x:c r="H7" s="55" t="str"/>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="55"/>
-      <x:c r="B8" s="55"/>
-      <x:c r="C8" s="55"/>
-      <x:c r="D8" s="55"/>
-      <x:c r="E8" s="55"/>
-      <x:c r="F8" s="55"/>
-      <x:c r="G8" s="55"/>
-      <x:c r="H8" s="55"/>
+    <x:row r="6" ht="96" hidden="0" customHeight="1">
+      <x:c r="A6" s="55" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="B6" s="55" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C6" s="55" t="str">
+        <x:v>聚焦首次启动与 Termux 后台常驻诊断体验</x:v>
+      </x:c>
+      <x:c r="D6" s="55" t="str">
+        <x:v>FirstTavernStartGuide、PermissionStatusSummary、LauncherHealthCheck、LukoaLauncherScreen 与相关测试</x:v>
+      </x:c>
+      <x:c r="E6" s="55" t="str">
+        <x:v>iQOO 首启提醒跳过条件依赖系统后台常驻检测，仍需真机确认不同系统返回是否准确。</x:v>
+      </x:c>
+      <x:c r="F6" s="55" t="str">
+        <x:v>是：单测、Kotlin 编译、Lint、Debug APK 均通过</x:v>
+      </x:c>
+      <x:c r="G6" s="55" t="str">
+        <x:v>按 v0.9.1-beta4 聚焦首次启动 + Termux 后台保活/诊断闭环。</x:v>
+      </x:c>
+      <x:c r="H6" s="55" t="str">
+        <x:v>恢复本次修改的代码和测试文件即可；未改发布脚本或数据迁移逻辑。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="80" hidden="0" customHeight="1">
+      <x:c r="A7" s="55" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="B7" s="55" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C7" s="55" t="str">
+        <x:v>减少首启引导重复弹出</x:v>
+      </x:c>
+      <x:c r="D7" s="55" t="str">
+        <x:v>FirstTavernStartGuide、FirstTavernStartGuideTest</x:v>
+      </x:c>
+      <x:c r="E7" s="55" t="str">
+        <x:v>成功历史依赖日志/状态文本识别，后续新增运行成功文案时要同步考虑。</x:v>
+      </x:c>
+      <x:c r="F7" s="55" t="str">
+        <x:v>是：单测、Kotlin 编译、Lint、Debug APK 均通过</x:v>
+      </x:c>
+      <x:c r="G7" s="55" t="str">
+        <x:v>继续优化首启 + 后台保活/诊断闭环，补 App 中文运行状态和 endpoint responding 标记。</x:v>
+      </x:c>
+      <x:c r="H7" s="55" t="str">
+        <x:v>恢复 FirstTavernStartGuide 和对应测试改动即可。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="140" hidden="0" customHeight="1">
+      <x:c r="A8" s="55" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="B8" s="55" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C8" s="55" t="str">
+        <x:v>优化 Termux 唤醒并返回与回前台复查链路</x:v>
+      </x:c>
+      <x:c r="D8" s="55" t="str">
+        <x:v>MainActivity、TermuxWakePolicy、启动页/首次引导、权限诊断与相关测试</x:v>
+      </x:c>
+      <x:c r="E8" s="55" t="str">
+        <x:v>Android 普通权限下无法可靠判断 Termux 是否已在前台或后台可见；本版改为按安装、RUN_COMMAND、后台常驻与冷却策略触发，仍需真机确认自动返回行为。</x:v>
+      </x:c>
+      <x:c r="F8" s="55" t="str">
+        <x:v>是：单测、全量单元、Kotlin、Lint、Debug/Release APK 通过；真机待测。</x:v>
+      </x:c>
+      <x:c r="G8" s="55" t="str">
+        <x:v>按用户要求优化“唤醒 Termux 并返回”和首次跳转 Termux 链路，回前台时条件复查并防止重复跳转。</x:v>
+      </x:c>
+      <x:c r="H8" s="55" t="str">
+        <x:v>回退 v0.9.1-beta5 提交/tag；或恢复本次唤醒策略、生命周期、UI 文案和测试改动。</x:v>
+      </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="55"/>

</xml_diff>

<commit_message>
Harden Termux wake retry handling
</commit_message>
<xml_diff>
--- a/docs/project-management/lukua-launcher-AI项目管理模板.xlsx
+++ b/docs/project-management/lukua-launcher-AI项目管理模板.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R0a9eb14720df4291"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总表" sheetId="2" r:id="R9383fa6503694b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发版检查" sheetId="3" r:id="R77492ed9b2304fcd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兼容性测试" sheetId="4" r:id="R76644b2741ec42f7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI协作记录" sheetId="5" r:id="Rb28bc6f2f7e04746"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="项目总览" sheetId="1" r:id="R72a76b9161394f9a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="版本总表" sheetId="2" r:id="Rcc01afd937fd44c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="发版检查" sheetId="3" r:id="R573286b3864340ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兼容性测试" sheetId="4" r:id="Rd768a902db63405b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI协作记录" sheetId="5" r:id="R63bfde379e3f47d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1162,7 +1162,7 @@
       </x:c>
       <x:c r="E11" s="56" t="n">
         <x:f>COUNTA('版本总表'!A6:A200)</x:f>
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1892,19 +1892,43 @@
         <x:v>发布为 prerelease，建议真机确认后继续作为主线。</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="55" t="str"/>
-      <x:c r="B7" s="55" t="str"/>
-      <x:c r="C7" s="55" t="str"/>
-      <x:c r="D7" s="55" t="str"/>
-      <x:c r="E7" s="55" t="str"/>
-      <x:c r="F7" s="55" t="str"/>
-      <x:c r="G7" s="55" t="str"/>
-      <x:c r="H7" s="55" t="str"/>
-      <x:c r="I7" s="55" t="str"/>
-      <x:c r="J7" s="55" t="str"/>
-      <x:c r="K7" s="55" t="str"/>
-      <x:c r="L7" s="55" t="str"/>
+    <x:row r="7" ht="72" hidden="0" customHeight="1">
+      <x:c r="A7" s="55" t="str">
+        <x:v>v0.9.1-beta6</x:v>
+      </x:c>
+      <x:c r="B7" s="55" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="C7" s="55" t="str">
+        <x:v>v0.9.1-beta5</x:v>
+      </x:c>
+      <x:c r="D7" s="55" t="str">
+        <x:v>beta</x:v>
+      </x:c>
+      <x:c r="E7" s="55" t="str">
+        <x:v>继续加固 Termux 唤醒和启动提示</x:v>
+      </x:c>
+      <x:c r="F7" s="55" t="str">
+        <x:v>唤醒冷却只在真正打开 Termux 后记录；启动命令已发但没自动打开 Termux 时，提示手动打开并不要重复点启动。</x:v>
+      </x:c>
+      <x:c r="G7" s="55" t="str">
+        <x:v>修复唤醒失败后仍进入冷却、导致用户短时间内无法重试且提示不准确的问题。</x:v>
+      </x:c>
+      <x:c r="H7" s="55" t="str">
+        <x:v>本环境无在线 adb 设备，仍需真机验证不同系统自动打开 Termux 的行为。</x:v>
+      </x:c>
+      <x:c r="I7" s="55" t="str">
+        <x:v>构建通过</x:v>
+      </x:c>
+      <x:c r="J7" s="55" t="str">
+        <x:v>构建通过，真机待测</x:v>
+      </x:c>
+      <x:c r="K7" s="55" t="str">
+        <x:v>是</x:v>
+      </x:c>
+      <x:c r="L7" s="55" t="str">
+        <x:v>发布为 prerelease，建议作为 beta5 后续修正版。</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="55" t="str"/>
@@ -5324,15 +5348,31 @@
         <x:v>回退 v0.9.1-beta5 提交/tag；或恢复本次唤醒策略、生命周期、UI 文案和测试改动。</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
-      <x:c r="A9" s="55"/>
-      <x:c r="B9" s="55"/>
-      <x:c r="C9" s="55"/>
-      <x:c r="D9" s="55"/>
-      <x:c r="E9" s="55"/>
-      <x:c r="F9" s="55"/>
-      <x:c r="G9" s="55"/>
-      <x:c r="H9" s="55"/>
+    <x:row r="9" ht="112" hidden="0" customHeight="1">
+      <x:c r="A9" s="55" t="str">
+        <x:v>2026-07-07</x:v>
+      </x:c>
+      <x:c r="B9" s="55" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+      <x:c r="C9" s="55" t="str">
+        <x:v>专项加固 Termux 唤醒失败重试与启动提示</x:v>
+      </x:c>
+      <x:c r="D9" s="55" t="str">
+        <x:v>LauncherStateStore、MainActivity、TavernController、StatusSummarizerTest</x:v>
+      </x:c>
+      <x:c r="E9" s="55" t="str">
+        <x:v>真机上仍需确认系统拒绝自动打开 Termux 时，用户手动打开 Termux 后启动日志是否持续可见。</x:v>
+      </x:c>
+      <x:c r="F9" s="55" t="str">
+        <x:v>是：全量单元、Kotlin、Lint、Debug APK、Release APK 通过；真机待测。</x:v>
+      </x:c>
+      <x:c r="G9" s="55" t="str">
+        <x:v>按用户要求继续检查 Termux 唤醒和启动酒馆链路，修复失败冷却占用并加固启动中状态摘要。</x:v>
+      </x:c>
+      <x:c r="H9" s="55" t="str">
+        <x:v>回退 v0.9.1-beta6 提交/tag；或恢复本次状态存储、唤醒调用、启动提示和测试改动。</x:v>
+      </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="55"/>

</xml_diff>